<commit_message>
battle map, world map fix
</commit_message>
<xml_diff>
--- a/Design/config/CityDevConfig.xlsx
+++ b/Design/config/CityDevConfig.xlsx
@@ -373,10 +373,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>50,250</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>3,9</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -402,6 +398,10 @@
   </si>
   <si>
     <t>-500,-1500</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>20,100</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -879,7 +879,7 @@
         <v>35</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>77</v>
@@ -1094,7 +1094,7 @@
         <v>50</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>53</v>
@@ -1136,13 +1136,13 @@
         <v>53</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>85</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
@@ -1178,7 +1178,7 @@
         <v>63</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
@@ -1214,7 +1214,7 @@
         <v>65</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
@@ -1256,13 +1256,13 @@
         <v>53</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="K11" s="6" t="s">
         <v>85</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M11" s="4" t="s">
         <v>73</v>

</xml_diff>